<commit_message>
feat(m5): add student application module and unit tests
</commit_message>
<xml_diff>
--- a/test-evidence/M5-Huang-Haoyu/UT-M5-table.xlsx
+++ b/test-evidence/M5-Huang-Haoyu/UT-M5-table.xlsx
@@ -514,12 +514,36 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>A student (ID=1) and an available ProjectTopic (ID=10) exist. Student has no existing applications.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>submitApplication(student, 10L, "I am interested")</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Application saved with pending status.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Application status is pending, personalStatement is "I am interested".</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Application status=pending, personalStatement="I am interested".</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -532,12 +556,36 @@
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>A student (ID=1) already has a pending application for ProjectTopic (ID=10).</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>submitApplication(student, 10L, "I am interested")</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Throws IllegalStateException.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>System throws IllegalStateException with message "You have already applied to this project."</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>IllegalStateException thrown with message "You have already applied to this project."</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -550,12 +598,36 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>A student (ID=1) has a pending application (ID=5) for a project.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>withdrawApplication(student, 5L)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Application status changed to withdrawn.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Application status changes from pending to withdrawn.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Application status=withdrawn.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -568,12 +640,36 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>A student (ID=1) has an accepted application (ID=5). Status is not pending.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>withdrawApplication(student, 5L)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Throws IllegalStateException.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>System throws IllegalStateException with message "Only pending applications can be withdrawn."</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>IllegalStateException thrown with message "Only pending applications can be withdrawn."</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
M5 student application Sprint 3
</commit_message>
<xml_diff>
--- a/test-evidence/M5-Huang-Haoyu/UT-M5-table.xlsx
+++ b/test-evidence/M5-Huang-Haoyu/UT-M5-table.xlsx
@@ -600,27 +600,27 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>A student (ID=1) has a pending application (ID=5) for a project.</t>
+          <t>A student is logged in. ProjectTopic (ID=1) exists.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>withdrawApplication(student, 5L)</t>
+          <t>POST /api/applications with projectId=1, personalStatement="too short" (less than 50 chars)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Application status changed to withdrawn.</t>
+          <t>HTTP 400 Bad Request.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Application status changes from pending to withdrawn.</t>
+          <t>Server returns 400 status with message "Personal statement must be at least 50 characters."</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Application status=withdrawn.</t>
+          <t>HTTP 400 returned with message "Personal statement must be at least 50 characters."</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -642,27 +642,27 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>A student (ID=1) has an accepted application (ID=5). Status is not pending.</t>
+          <t>A student is logged in and already has a pending application for ProjectTopic (ID=1).</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>withdrawApplication(student, 5L)</t>
+          <t>POST /api/applications with projectId=1, personalStatement (50+ chars)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Throws IllegalStateException.</t>
+          <t>HTTP 409 Conflict.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>System throws IllegalStateException with message "Only pending applications can be withdrawn."</t>
+          <t>Server returns 409 status with message "You have already applied to this project."</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>IllegalStateException thrown with message "Only pending applications can be withdrawn."</t>
+          <t>HTTP 409 returned with message "You have already applied to this project."</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">

</xml_diff>